<commit_message>
collection of small code updates for more practical use
</commit_message>
<xml_diff>
--- a/2_REVUB_control_files/parameters_simulation.xlsx
+++ b/2_REVUB_control_files/parameters_simulation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/REVUB code repo/2_REVUB_control_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="807" documentId="13_ncr:1_{3E75B3F6-DB26-4BD5-A9C7-B5D5CA9FF346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12BC7E3D-FB24-4E8F-A48D-DA7EF620EDBA}"/>
+  <xr:revisionPtr revIDLastSave="808" documentId="13_ncr:1_{3E75B3F6-DB26-4BD5-A9C7-B5D5CA9FF346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CB1F492-1DBB-4CA3-917F-A710347EFE07}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{B27AEA38-A928-4B6A-AF9B-7A28216807AA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{B27AEA38-A928-4B6A-AF9B-7A28216807AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Hydropower plant parameters" sheetId="2" r:id="rId1"/>
@@ -376,9 +376,6 @@
     <t>prevent_droughts_increase</t>
   </si>
   <si>
-    <t>select this option to discard potential solutions in which hydropower blackouts are worse under BAL/STOR than under CONV (0 = not prevented, 1 = prevented)</t>
-  </si>
-  <si>
     <t>name of corresponding worksheet in the "data" Excel sheets from which to pull data (hourly solar CF as fraction/percentage; hours in rows, years in columns); leave empty if scenario has no solar</t>
   </si>
   <si>
@@ -707,6 +704,9 @@
       </rPr>
       <t>In case this HPP is the principal flexibility provider in a cascade, and there is a hydropower plant upstream with reservoir that serves both plants, insert here the share of volume changes allocated to the upper reservoir.</t>
     </r>
+  </si>
+  <si>
+    <t>select this option to discard potential solutions in which hydropower blackouts are worse under BAL/STOR than under CONV (0 = not prevented, 1 = prevented) [only during calibration period]</t>
   </si>
 </sst>
 </file>
@@ -927,10 +927,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1240,7 +1236,7 @@
   <sheetData>
     <row r="1" spans="1:16" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B1" s="7"/>
     </row>
@@ -1252,13 +1248,13 @@
         <v>16</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>135</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:16" s="10" customFormat="1" x14ac:dyDescent="0.35">
@@ -1280,38 +1276,38 @@
     </row>
     <row r="4" spans="1:16" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A4" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B4" s="7"/>
     </row>
     <row r="5" spans="1:16" s="6" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:16" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="P6" s="12"/>
     </row>
     <row r="7" spans="1:16" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="8" spans="1:16" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A8" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B8" s="7"/>
     </row>
@@ -1325,10 +1321,10 @@
     </row>
     <row r="10" spans="1:16" s="3" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="11" spans="1:16" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -1336,7 +1332,7 @@
         <v>25</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" spans="1:16" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -1344,7 +1340,7 @@
         <v>24</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="13" spans="1:16" s="3" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1352,7 +1348,7 @@
         <v>21</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:16" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -1360,7 +1356,7 @@
         <v>22</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:16" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -1368,7 +1364,7 @@
         <v>23</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" spans="1:16" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
@@ -1381,7 +1377,7 @@
     </row>
     <row r="17" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A17" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B17" s="7"/>
     </row>
@@ -1395,7 +1391,7 @@
     </row>
     <row r="19" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A19" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B19" s="7"/>
     </row>
@@ -1404,12 +1400,12 @@
         <v>30</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="21" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A21" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B21" s="7"/>
     </row>
@@ -1466,7 +1462,7 @@
         <v>45</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="29" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1575,7 +1571,7 @@
     </row>
     <row r="42" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A42" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B42" s="7"/>
     </row>
@@ -1584,7 +1580,7 @@
         <v>92</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="44" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
@@ -1592,12 +1588,12 @@
         <v>93</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="45" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A45" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B45" s="7"/>
     </row>
@@ -1606,7 +1602,7 @@
         <v>81</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="47" spans="1:2" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -1614,7 +1610,7 @@
         <v>82</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="48" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
@@ -1622,7 +1618,7 @@
         <v>83</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="49" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
@@ -1630,12 +1626,12 @@
         <v>84</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="50" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A50" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B50" s="7"/>
     </row>
@@ -1644,7 +1640,7 @@
         <v>71</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="52" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1652,7 +1648,7 @@
         <v>72</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="53" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1660,7 +1656,7 @@
         <v>73</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="54" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1668,7 +1664,7 @@
         <v>74</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="55" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1676,7 +1672,7 @@
         <v>75</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="56" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1684,12 +1680,12 @@
         <v>76</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="57" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A57" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B57" s="7"/>
     </row>
@@ -1698,7 +1694,7 @@
         <v>85</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="59" spans="1:2" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -1706,7 +1702,7 @@
         <v>86</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="60" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
@@ -1714,7 +1710,7 @@
         <v>87</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="61" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
@@ -1722,7 +1718,7 @@
         <v>88</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1842,13 +1838,13 @@
     </row>
     <row r="10" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B10" s="2">
         <v>2</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="29" x14ac:dyDescent="0.35">
@@ -1870,7 +1866,7 @@
         <v>1</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>95</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="29" x14ac:dyDescent="0.35">
@@ -1892,7 +1888,7 @@
         <v>0</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new extended training dataset updated to version 1.1; merged master files for simulation and plotting
</commit_message>
<xml_diff>
--- a/2_REVUB_control_files/parameters_simulation.xlsx
+++ b/2_REVUB_control_files/parameters_simulation.xlsx
@@ -8,15 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/REVUB code repo/2_REVUB_control_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="808" documentId="13_ncr:1_{3E75B3F6-DB26-4BD5-A9C7-B5D5CA9FF346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CB1F492-1DBB-4CA3-917F-A710347EFE07}"/>
+  <xr:revisionPtr revIDLastSave="1137" documentId="13_ncr:1_{3E75B3F6-DB26-4BD5-A9C7-B5D5CA9FF346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0401A84F-0CE9-4586-9401-3AB241E8D865}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{B27AEA38-A928-4B6A-AF9B-7A28216807AA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="735" xr2:uid="{B27AEA38-A928-4B6A-AF9B-7A28216807AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Hydropower plant parameters" sheetId="2" r:id="rId1"/>
     <sheet name="General parameters" sheetId="3" r:id="rId2"/>
+    <sheet name="Plot power output (single HPP)" sheetId="4" r:id="rId3"/>
+    <sheet name="Plot power output (multi HPP)" sheetId="6" r:id="rId4"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Plot power output (single HPP)'!$A$1:$C$16</definedName>
     <definedName name="g">'General parameters'!$B$5</definedName>
     <definedName name="HPP_name">'Hydropower plant parameters'!$C$2:$XFD$2</definedName>
     <definedName name="LOEE_allowed">'General parameters'!$B$8</definedName>
@@ -47,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="206">
   <si>
     <t>year_start</t>
   </si>
@@ -158,9 +161,6 @@
   </si>
   <si>
     <t>maximum lake volume in m^3</t>
-  </si>
-  <si>
-    <t>V_initial_frac</t>
   </si>
   <si>
     <t>initial filling fraction of lake volume</t>
@@ -580,15 +580,6 @@
     <t>wish to activate pumped storage module STOR (Note 7) for at least one hydropower plant or not? (0 = no, 1 = yes)</t>
   </si>
   <si>
-    <t>[name 1]</t>
-  </si>
-  <si>
-    <t>[name 2]</t>
-  </si>
-  <si>
-    <t>[name 3]</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">turbine efficiency as fraction </t>
     </r>
@@ -706,14 +697,366 @@
     </r>
   </si>
   <si>
+    <t>f_initial_frac</t>
+  </si>
+  <si>
     <t>select this option to discard potential solutions in which hydropower blackouts are worse under BAL/STOR than under CONV (0 = not prevented, 1 = prevented) [only during calibration period]</t>
+  </si>
+  <si>
+    <t>plot_HPP</t>
+  </si>
+  <si>
+    <t>exact name of hydropower plant to plot</t>
+  </si>
+  <si>
+    <t>plot_year</t>
+  </si>
+  <si>
+    <t>for monthly and hourly graphs: choose which simulation year to take (1 = first year; 2 = second year; etc.)</t>
+  </si>
+  <si>
+    <t>plot_month</t>
+  </si>
+  <si>
+    <t>for hourly graph: choose month to plot (1 = Jan; 2 = Feb; etc.)</t>
+  </si>
+  <si>
+    <t>plot_day_month</t>
+  </si>
+  <si>
+    <t>for hourly graph: choose day of the month that the plot starts with</t>
+  </si>
+  <si>
+    <t>plot_num_days</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">for hourly graph: number of days to show, starting at </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>plot_day_month</t>
+    </r>
+  </si>
+  <si>
+    <t>plot_RoR_part</t>
+  </si>
+  <si>
+    <t>set to 1 to plot run-of-river component of electricity generation, or to 0 to leave out this component</t>
+  </si>
+  <si>
+    <t>plot_ELCC_line</t>
+  </si>
+  <si>
+    <t>set to 1 to include a bold black line for ELCC, or to 0 to leave out</t>
+  </si>
+  <si>
+    <t>Figure1_on</t>
+  </si>
+  <si>
+    <t>set to 1 to plot bathymetry relations, or to 0 to turn off</t>
+  </si>
+  <si>
+    <t>Figure2_on</t>
+  </si>
+  <si>
+    <t>set to 1 to plot hydraulic head and inflow/outflow IQ ranges, or to 0 to turn off</t>
+  </si>
+  <si>
+    <t>Figure3_on</t>
+  </si>
+  <si>
+    <t>set to 1 to plot full time series of reservoir volume and inflow/outflow, or to 0 to turn off</t>
+  </si>
+  <si>
+    <t>Figure4_on</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">set to 1 to plot month-by-month power generation in year defined by </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>plot_year</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, or to 0 to turn off</t>
+    </r>
+  </si>
+  <si>
+    <t>Figure5_on</t>
+  </si>
+  <si>
+    <t>set to 1 to plot year-by-year power generation, or to 0 to turn off</t>
+  </si>
+  <si>
+    <t>Figure6_on</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">set to 1 to plot hourly power generation from date </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>plot_day_month/plot_month/plot_year</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> for number of days = </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>plot_num_days</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, or to 0 to turn off</t>
+    </r>
+  </si>
+  <si>
+    <t>Figure7_on</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">set to 1 to plot regulated reservoir release statistics [see worksheet </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Plot release rules (single HPP)]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, or to 0 to turn off </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[Note: currently only available for BAL]</t>
+    </r>
+  </si>
+  <si>
+    <t>Figure8_on</t>
+  </si>
+  <si>
+    <t>set to 1 to plot hydroturbine use statistics, or to 0 to turn off</t>
+  </si>
+  <si>
+    <t>Figure9_on</t>
+  </si>
+  <si>
+    <r>
+      <t>set to 1 to plot operational regime statistics, or to 0 to turn off [</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Note: currently only available for BAL</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>]</t>
+    </r>
+  </si>
+  <si>
+    <t>plot_rules_month</t>
+  </si>
+  <si>
+    <t>plot_rules_hr</t>
+  </si>
+  <si>
+    <t>enter the names of the hydropower plants to include in this plot in row 2, starting in column B</t>
+  </si>
+  <si>
+    <t>plot_HPP_multiple</t>
+  </si>
+  <si>
+    <t>[choose] whether to use static (=0; same year-to-year) or dynamic (=1; time series) demand and capacity</t>
+  </si>
+  <si>
+    <t>choose_demand_type</t>
+  </si>
+  <si>
+    <t>[static: demand]</t>
+  </si>
+  <si>
+    <t>P_total_av</t>
+  </si>
+  <si>
+    <t>total average load (MW) assumed for graph of full power mix</t>
+  </si>
+  <si>
+    <t>[static: non-hydro capacity]</t>
+  </si>
+  <si>
+    <t>P_r_total_thermal</t>
+  </si>
+  <si>
+    <t>total flexible non-hydro (thermal, importc, &amp;c.) capacity assumed available (MW)</t>
+  </si>
+  <si>
+    <t>[dynamic: demand] enter a time series of average demand (MW) for each year in the simulation</t>
+  </si>
+  <si>
+    <t>[year 1]</t>
+  </si>
+  <si>
+    <t>[year 2]</t>
+  </si>
+  <si>
+    <t>&amp;c…</t>
+  </si>
+  <si>
+    <t>P_total_av_series</t>
+  </si>
+  <si>
+    <t>[dynamic: non-hydro capacity] enter a time series of available capacity (MW) of flexible non-hydro assets (thermal, imports, &amp;c.)</t>
+  </si>
+  <si>
+    <t>P_r_total_thermal_series</t>
+  </si>
+  <si>
+    <t>[plotting] set visualisation parameters</t>
+  </si>
+  <si>
+    <t>plot_year_multiple</t>
+  </si>
+  <si>
+    <t>plot_month_multiple</t>
+  </si>
+  <si>
+    <t>plot_day_month_multiple</t>
+  </si>
+  <si>
+    <t>plot_num_days_multiple</t>
+  </si>
+  <si>
+    <t>plot_ramping_range</t>
+  </si>
+  <si>
+    <t>number of hours to include in ramping envelopes</t>
+  </si>
+  <si>
+    <t>chosen_load</t>
+  </si>
+  <si>
+    <t>enter here the name of the target load curve to be used for the plot</t>
+  </si>
+  <si>
+    <t>plot_ELCC_line_multiple</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">in this row, enter all months (using numbers 1-12, one per cell) for which to plot release rules (Figure 7) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>→</t>
+    </r>
+  </si>
+  <si>
+    <t>in this row, enter all hours of the day (using numbers 0-23, one per cell) for which to plot release rules (Figure 7) →</t>
+  </si>
+  <si>
+    <t>[name 1]</t>
+  </si>
+  <si>
+    <t>[name 2]</t>
+  </si>
+  <si>
+    <t>[name 3]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0E+00"/>
+  </numFmts>
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -792,6 +1135,27 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -883,12 +1247,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -910,8 +1275,19 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="3" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
+    <cellStyle name="Explanatory Text" xfId="3" builtinId="53"/>
     <cellStyle name="Input" xfId="1" builtinId="20"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Note" xfId="2" builtinId="10"/>
@@ -1226,21 +1602,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10D23870-37A0-4EFA-BF75-9E0BBC5C39B4}">
-  <dimension ref="A1:P61"/>
+  <dimension ref="A1:M61"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.81640625" style="5" customWidth="1"/>
     <col min="2" max="2" width="71.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="15" customWidth="1"/>
+    <col min="3" max="5" width="9.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:13" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B1" s="7"/>
     </row>
-    <row r="2" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>15</v>
       </c>
@@ -1248,70 +1624,61 @@
         <v>16</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>133</v>
+        <v>203</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>134</v>
+        <v>204</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" s="10" customFormat="1" x14ac:dyDescent="0.35">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>17</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="10">
-        <v>0</v>
-      </c>
-      <c r="D3" s="10">
-        <v>0</v>
-      </c>
-      <c r="E3" s="10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
+    </row>
+    <row r="4" spans="1:13" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A4" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B4" s="7"/>
     </row>
-    <row r="5" spans="1:16" s="6" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" s="6" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A6" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="M6" s="12"/>
+    </row>
+    <row r="7" spans="1:13" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A7" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
-      <c r="A6" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="P6" s="12"/>
-    </row>
-    <row r="7" spans="1:16" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
-      <c r="A7" s="5" t="s">
-        <v>124</v>
-      </c>
       <c r="B7" s="1" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A8" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B8" s="7"/>
     </row>
-    <row r="9" spans="1:16" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>19</v>
       </c>
@@ -1319,55 +1686,55 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:16" s="3" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" s="3" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>25</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" s="3" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" s="3" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>21</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>22</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
         <v>26</v>
       </c>
@@ -1375,13 +1742,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:4" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A17" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B17" s="7"/>
     </row>
-    <row r="18" spans="1:2" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
         <v>28</v>
       </c>
@@ -1389,43 +1756,44 @@
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:4" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A19" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B19" s="7"/>
     </row>
-    <row r="20" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
         <v>30</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A21" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B21" s="7"/>
     </row>
-    <row r="22" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="23" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
         <v>35</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D23" s="13"/>
+    </row>
+    <row r="24" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>33</v>
       </c>
@@ -1433,7 +1801,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="25" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
         <v>31</v>
       </c>
@@ -1441,284 +1809,284 @@
         <v>32</v>
       </c>
     </row>
-    <row r="26" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B26" s="1" t="s">
+    </row>
+    <row r="27" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="5" t="s">
+      <c r="B27" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B27" s="1" t="s">
+    </row>
+    <row r="28" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="5" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="5" t="s">
+      <c r="B28" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="5" t="s">
+      <c r="B30" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B30" s="1" t="s">
+    </row>
+    <row r="31" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="5" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="5" t="s">
+      <c r="B31" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B31" s="1" t="s">
+    </row>
+    <row r="32" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="5" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="5" t="s">
+      <c r="B32" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="33" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="34" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="35" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="36" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="37" spans="1:2" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="38" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="39" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="40" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="41" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="42" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A42" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B42" s="7"/>
     </row>
     <row r="43" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="44" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="45" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A45" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B45" s="7"/>
     </row>
     <row r="46" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="47" spans="1:2" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="48" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="49" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="50" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A50" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B50" s="7"/>
     </row>
     <row r="51" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="52" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="53" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="54" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="55" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="56" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="57" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A57" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B57" s="7"/>
     </row>
     <row r="58" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="59" spans="1:2" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="60" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="61" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -1794,13 +2162,13 @@
     </row>
     <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B6" s="2">
         <v>90</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="58" x14ac:dyDescent="0.35">
@@ -1827,57 +2195,57 @@
     </row>
     <row r="9" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B9" s="2">
         <v>1000</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B10" s="2">
         <v>2</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B11" s="2">
         <v>0</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B12" s="2">
         <v>1</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B13" s="2">
         <v>0</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="29" x14ac:dyDescent="0.35">
@@ -1888,10 +2256,412 @@
         <v>0</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE0C23C7-BBBB-4B68-BF11-FAE50DD24DE8}">
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>148</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>150</v>
+      </c>
+      <c r="B6" s="15"/>
+      <c r="C6" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B7" s="15"/>
+      <c r="C7" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>154</v>
+      </c>
+      <c r="B8" s="15"/>
+      <c r="C8" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" s="15"/>
+      <c r="C9" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>158</v>
+      </c>
+      <c r="B10" s="15"/>
+      <c r="C10" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>160</v>
+      </c>
+      <c r="B11" s="15"/>
+      <c r="C11" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>162</v>
+      </c>
+      <c r="B12" s="15"/>
+      <c r="C12" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>164</v>
+      </c>
+      <c r="B13" s="15"/>
+      <c r="C13" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>166</v>
+      </c>
+      <c r="B14" s="15"/>
+      <c r="C14" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>168</v>
+      </c>
+      <c r="B15" s="15"/>
+      <c r="C15" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>170</v>
+      </c>
+      <c r="B16" s="15"/>
+      <c r="C16" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B18" s="16" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B20" s="16" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>173</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1" xr:uid="{74C14F83-5E40-41AC-B7F9-E4A97E0F6335}">
+      <formula1>HPP_name</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25702544-B17E-4AFF-8FD3-F5A17DC2467E}">
+  <dimension ref="A1:O28"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="23.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.453125" customWidth="1"/>
+    <col min="3" max="3" width="12.7265625" customWidth="1"/>
+    <col min="4" max="4" width="11.7265625" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B1" s="16" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B4" s="16" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B5" s="15"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B7" s="16" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B10" s="16" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>182</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B13" s="16" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B14" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+    </row>
+    <row r="15" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>188</v>
+      </c>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="12"/>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12"/>
+      <c r="O15" s="18"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B17" s="16" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B18" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+    </row>
+    <row r="19" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>190</v>
+      </c>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="12"/>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12"/>
+      <c r="O19" s="12"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B21" s="16" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>192</v>
+      </c>
+      <c r="B22" s="2"/>
+      <c r="C22" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>193</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>194</v>
+      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>195</v>
+      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>196</v>
+      </c>
+      <c r="B26" s="2"/>
+      <c r="C26" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>198</v>
+      </c>
+      <c r="B27" s="14"/>
+      <c r="C27" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>200</v>
+      </c>
+      <c r="B28" s="15"/>
+      <c r="C28" t="s">
+        <v>153</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:XFD2" xr:uid="{5A1F5E20-D18E-45C4-BD57-D29767579F5A}">
+      <formula1>HPP_name</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
harmonising nomenclature between Manual and training material
</commit_message>
<xml_diff>
--- a/2_REVUB_control_files/parameters_simulation.xlsx
+++ b/2_REVUB_control_files/parameters_simulation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/REVUB code repo/2_REVUB_control_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1137" documentId="13_ncr:1_{3E75B3F6-DB26-4BD5-A9C7-B5D5CA9FF346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0401A84F-0CE9-4586-9401-3AB241E8D865}"/>
+  <xr:revisionPtr revIDLastSave="1141" documentId="13_ncr:1_{3E75B3F6-DB26-4BD5-A9C7-B5D5CA9FF346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8F75BF1-756E-4023-AE5F-B2652570C564}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="735" xr2:uid="{B27AEA38-A928-4B6A-AF9B-7A28216807AA}"/>
   </bookViews>
@@ -577,9 +577,6 @@
     <t>Number of loops for iterative estimation of P_stable in BAL/STOR (see eq. S9 &amp; explanation below eq. S19). Usually, 2 suffices; use 1 for quicker (but less accurate) simulations.</t>
   </si>
   <si>
-    <t>wish to activate pumped storage module STOR (Note 7) for at least one hydropower plant or not? (0 = no, 1 = yes)</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">turbine efficiency as fraction </t>
     </r>
@@ -1047,6 +1044,9 @@
   </si>
   <si>
     <t>[name 3]</t>
+  </si>
+  <si>
+    <t>wish to activate pumped storage module STOR (cf. Manual, Note 6) for at least one hydropower plant or not? (0 = no, 1 = yes)</t>
   </si>
 </sst>
 </file>
@@ -1624,13 +1624,13 @@
         <v>16</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>204</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="3" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.35">
@@ -1657,10 +1657,10 @@
     </row>
     <row r="6" spans="1:13" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="M6" s="12"/>
     </row>
@@ -1669,7 +1669,7 @@
         <v>123</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:13" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
@@ -1688,10 +1688,10 @@
     </row>
     <row r="10" spans="1:13" s="3" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="11" spans="1:13" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -1830,12 +1830,12 @@
         <v>44</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="29" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>37</v>
@@ -2234,7 +2234,7 @@
         <v>1</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="29" x14ac:dyDescent="0.35">
@@ -2256,7 +2256,7 @@
         <v>0</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>131</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -2275,166 +2275,166 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B6" s="15"/>
       <c r="C6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B7" s="15"/>
       <c r="C7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B8" s="15"/>
       <c r="C8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B10" s="15"/>
       <c r="C10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B12" s="15"/>
       <c r="C12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B13" s="15"/>
       <c r="C13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B14" s="15"/>
       <c r="C14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B15" s="15"/>
       <c r="C15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B16" s="15"/>
       <c r="C16" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B18" s="16" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="19" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B20" s="16" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="21" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -2462,67 +2462,67 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B1" s="16" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="2" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B4" s="16" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B5" s="15"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B7" s="16" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B10" s="16" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B13" s="16" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B14" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="C14" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="D14" s="17" t="s">
         <v>186</v>
-      </c>
-      <c r="D14" s="17" t="s">
-        <v>187</v>
       </c>
       <c r="E14" s="17"/>
       <c r="F14" s="17"/>
@@ -2531,7 +2531,7 @@
     </row>
     <row r="15" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
@@ -2550,18 +2550,18 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B17" s="16" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B18" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="C18" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="D18" s="17" t="s">
         <v>186</v>
-      </c>
-      <c r="D18" s="17" t="s">
-        <v>187</v>
       </c>
       <c r="E18" s="17"/>
       <c r="F18" s="17"/>
@@ -2570,7 +2570,7 @@
     </row>
     <row r="19" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
@@ -2589,70 +2589,70 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B21" s="16" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B27" s="14"/>
       <c r="C27" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B28" s="15"/>
       <c r="C28" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>